<commit_message>
Update fitur retrain dan prediksi
</commit_message>
<xml_diff>
--- a/static/hasil/data_prediksi.xlsx
+++ b/static/hasil/data_prediksi.xlsx
@@ -607,27 +607,25 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>87.39</v>
+        <v>57.94</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>23.84</v>
+        <v>33.32</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>5.7</v>
+        <v>11.63</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>4.54</v>
+        <v>2.85</v>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Buruk</t>
+          <t>Baik</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Kelembapan buruk, karena melebihi batas ideal dan dapat mengganggu pertumbuhan.
-Suhu buruk, karena terlalu rendah dari kisaran optimal.
-Penyinaran buruk, karena terlalu singkat untuk fotosintesis optimal.</t>
+          <t>Kelembapan udara baik, karena berada dalam kisaran optimal.</t>
         </is>
       </c>
     </row>
@@ -643,27 +641,26 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>86.83</v>
+        <v>59.08</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>23.84</v>
+        <v>27.67</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>5.41</v>
+        <v>12.2</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>4.8</v>
+        <v>3.01</v>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Buruk</t>
+          <t>Baik</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Kelembapan buruk, karena melebihi batas ideal dan dapat mengganggu pertumbuhan.
-Suhu buruk, karena terlalu rendah dari kisaran optimal.
-Penyinaran buruk, karena terlalu singkat untuk fotosintesis optimal.</t>
+          <t>Kelembapan udara baik, karena berada dalam kisaran optimal.
+Suhu udara baik, karena berada dalam kisaran optimal.</t>
         </is>
       </c>
     </row>
@@ -679,27 +676,26 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>86.17</v>
+        <v>59.64</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>23.83</v>
+        <v>26.25</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>4.53</v>
+        <v>12.47</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>5.04</v>
+        <v>3.21</v>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Buruk</t>
+          <t>Baik</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Kelembapan buruk, karena melebihi batas ideal dan dapat mengganggu pertumbuhan.
-Suhu buruk, karena terlalu rendah dari kisaran optimal.
-Penyinaran buruk, karena terlalu singkat untuk fotosintesis optimal.</t>
+          <t>Kelembapan udara baik, karena berada dalam kisaran optimal.
+Suhu udara baik, karena berada dalam kisaran optimal.</t>
         </is>
       </c>
     </row>
@@ -715,27 +711,26 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>85.56</v>
+        <v>62.63</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>23.83</v>
+        <v>26.75</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>3.66</v>
+        <v>12.23</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>5.19</v>
+        <v>3.43</v>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Buruk</t>
+          <t>Baik</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>Kelembapan buruk, karena melebihi batas ideal dan dapat mengganggu pertumbuhan.
-Suhu buruk, karena terlalu rendah dari kisaran optimal.
-Penyinaran buruk, karena terlalu singkat untuk fotosintesis optimal.</t>
+          <t>Kelembapan udara baik, karena berada dalam kisaran optimal.
+Suhu udara baik, karena berada dalam kisaran optimal.</t>
         </is>
       </c>
     </row>
@@ -751,16 +746,16 @@
         </is>
       </c>
       <c r="C11" s="5" t="n">
-        <v>84.95999999999999</v>
+        <v>68.14</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>23.81</v>
+        <v>27.92</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>3.37</v>
+        <v>11.38</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>5.27</v>
+        <v>3.65</v>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
@@ -769,8 +764,8 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Kelembapan baik, karena berada dalam kisaran optimal (50–85%).
-Curah hujan baik, karena memadai dalam batas ideal (2,6–8 mm).</t>
+          <t>Kelembapan udara baik, karena berada dalam kisaran optimal.
+Suhu udara baik, karena berada dalam kisaran optimal.</t>
         </is>
       </c>
     </row>
@@ -786,16 +781,16 @@
         </is>
       </c>
       <c r="C12" s="5" t="n">
-        <v>84.23999999999999</v>
+        <v>73.51000000000001</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>23.84</v>
+        <v>27.05</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>3.51</v>
+        <v>10.35</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>5.27</v>
+        <v>3.85</v>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
@@ -804,8 +799,8 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>Kelembapan baik, karena berada dalam kisaran optimal (50–85%).
-Curah hujan baik, karena memadai dalam batas ideal (2,6–8 mm).</t>
+          <t>Kelembapan udara baik, karena berada dalam kisaran optimal.
+Suhu udara baik, karena berada dalam kisaran optimal.</t>
         </is>
       </c>
     </row>
@@ -821,16 +816,16 @@
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>83.36</v>
+        <v>80.23</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>23.98</v>
+        <v>26.05</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>3.92</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>5.22</v>
+        <v>4.02</v>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
@@ -839,8 +834,8 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Kelembapan baik, karena berada dalam kisaran optimal (50–85%).
-Curah hujan baik, karena memadai dalam batas ideal (2,6–8 mm).</t>
+          <t>Kelembapan udara baik, karena berada dalam kisaran optimal.
+Suhu udara baik, karena berada dalam kisaran optimal.</t>
         </is>
       </c>
     </row>

</xml_diff>